<commit_message>
working two stage, error fixed
</commit_message>
<xml_diff>
--- a/Two Stage Deterministic equivalent/random_normal_forecast_data.xlsx
+++ b/Two Stage Deterministic equivalent/random_normal_forecast_data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Desktop/Vaccine_Tender/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Desktop/Vaccine_Tender/Two Stage Deterministic equivalent/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F1A34A30-8D23-4614-BCFD-51B5FDA2F136}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="8_{F1A34A30-8D23-4614-BCFD-51B5FDA2F136}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{54DB8D08-6987-438A-89C0-4E50DC93CC02}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{A5115543-AC87-4E62-8A65-1522949D5C3B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="9" xr2:uid="{A5115543-AC87-4E62-8A65-1522949D5C3B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,11 @@
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
     <sheet name="Sheet4" sheetId="4" r:id="rId4"/>
     <sheet name="Sheet5" sheetId="5" r:id="rId5"/>
+    <sheet name="Sheet6" sheetId="6" r:id="rId6"/>
+    <sheet name="Sheet7" sheetId="7" r:id="rId7"/>
+    <sheet name="Sheet8" sheetId="8" r:id="rId8"/>
+    <sheet name="Sheet9" sheetId="9" r:id="rId9"/>
+    <sheet name="Sheet10" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="12">
   <si>
     <t>PCV</t>
   </si>
@@ -907,6 +912,468 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5904865-E606-489B-B449-E4BD925F4A4E}">
+  <dimension ref="A1:K13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B1">
+        <v>1</v>
+      </c>
+      <c r="C1">
+        <v>2</v>
+      </c>
+      <c r="D1">
+        <v>3</v>
+      </c>
+      <c r="E1">
+        <v>4</v>
+      </c>
+      <c r="F1">
+        <v>5</v>
+      </c>
+      <c r="G1">
+        <v>6</v>
+      </c>
+      <c r="H1">
+        <v>7</v>
+      </c>
+      <c r="I1">
+        <v>8</v>
+      </c>
+      <c r="J1">
+        <v>9</v>
+      </c>
+      <c r="K1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2">
+        <v>415609019.04617053</v>
+      </c>
+      <c r="C2">
+        <v>382796030.65416956</v>
+      </c>
+      <c r="D2">
+        <v>919869439.18637204</v>
+      </c>
+      <c r="E2">
+        <v>154608386.45836771</v>
+      </c>
+      <c r="F2">
+        <v>602116627.59758711</v>
+      </c>
+      <c r="G2">
+        <v>749899819.97235596</v>
+      </c>
+      <c r="H2">
+        <v>836352851.17984498</v>
+      </c>
+      <c r="I2">
+        <v>875269871.35862076</v>
+      </c>
+      <c r="J2">
+        <v>940024211.45830357</v>
+      </c>
+      <c r="K2">
+        <v>733277731.44407725</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>26791240.142195012</v>
+      </c>
+      <c r="C3">
+        <v>38689169.944861226</v>
+      </c>
+      <c r="D3">
+        <v>34039132.651055574</v>
+      </c>
+      <c r="E3">
+        <v>26877974.901466619</v>
+      </c>
+      <c r="F3">
+        <v>46881340.138904341</v>
+      </c>
+      <c r="G3">
+        <v>47177018.392687067</v>
+      </c>
+      <c r="H3">
+        <v>73775600.009666696</v>
+      </c>
+      <c r="I3">
+        <v>74484333.971165538</v>
+      </c>
+      <c r="J3">
+        <v>56527699.736730404</v>
+      </c>
+      <c r="K3">
+        <v>77924603.592910603</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
+        <v>190948844.07116279</v>
+      </c>
+      <c r="C4">
+        <v>574271673.70995557</v>
+      </c>
+      <c r="D4">
+        <v>508106843.54881513</v>
+      </c>
+      <c r="E4">
+        <v>358734306.13637894</v>
+      </c>
+      <c r="F4">
+        <v>339540652.61159468</v>
+      </c>
+      <c r="G4">
+        <v>588101691.70337486</v>
+      </c>
+      <c r="H4">
+        <v>707887657.59311903</v>
+      </c>
+      <c r="I4">
+        <v>301070887.69854683</v>
+      </c>
+      <c r="J4">
+        <v>507470696.00852042</v>
+      </c>
+      <c r="K4">
+        <v>868142342.30724955</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5">
+        <v>545886518.23867655</v>
+      </c>
+      <c r="C5">
+        <v>678726381.22116768</v>
+      </c>
+      <c r="D5">
+        <v>734290499.30955684</v>
+      </c>
+      <c r="E5">
+        <v>719200133.09411359</v>
+      </c>
+      <c r="F5">
+        <v>604347397.85308969</v>
+      </c>
+      <c r="G5">
+        <v>1460640716.6727061</v>
+      </c>
+      <c r="H5">
+        <v>1222658755.0402675</v>
+      </c>
+      <c r="I5">
+        <v>1294822890.6755817</v>
+      </c>
+      <c r="J5">
+        <v>1108422810.5878639</v>
+      </c>
+      <c r="K5">
+        <v>1421683508.03038</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6">
+        <v>570605073.91759527</v>
+      </c>
+      <c r="C6">
+        <v>661397242.07395899</v>
+      </c>
+      <c r="D6">
+        <v>551049558.58273554</v>
+      </c>
+      <c r="E6">
+        <v>729467505.08887362</v>
+      </c>
+      <c r="F6">
+        <v>852703034.15588212</v>
+      </c>
+      <c r="G6">
+        <v>675272361.62296128</v>
+      </c>
+      <c r="H6">
+        <v>596442954.70324564</v>
+      </c>
+      <c r="I6">
+        <v>603390078.92934215</v>
+      </c>
+      <c r="J6">
+        <v>720240666.25842512</v>
+      </c>
+      <c r="K6">
+        <v>638491395.95045185</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>375139522.67123127</v>
+      </c>
+      <c r="C7">
+        <v>369688337.68584186</v>
+      </c>
+      <c r="D7">
+        <v>437276119.25633711</v>
+      </c>
+      <c r="E7">
+        <v>444592230.52522165</v>
+      </c>
+      <c r="F7">
+        <v>312002190.95961249</v>
+      </c>
+      <c r="G7">
+        <v>369142320.0867545</v>
+      </c>
+      <c r="H7">
+        <v>395672073.68059427</v>
+      </c>
+      <c r="I7">
+        <v>344527980.82132643</v>
+      </c>
+      <c r="J7">
+        <v>394175481.75587392</v>
+      </c>
+      <c r="K7">
+        <v>422270657.59424824</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8">
+        <v>449867903.82097661</v>
+      </c>
+      <c r="C8">
+        <v>371021724.53464144</v>
+      </c>
+      <c r="D8">
+        <v>307648881.91826731</v>
+      </c>
+      <c r="E8">
+        <v>457079487.18215239</v>
+      </c>
+      <c r="F8">
+        <v>262253010.64244753</v>
+      </c>
+      <c r="G8">
+        <v>565381184.93855238</v>
+      </c>
+      <c r="H8">
+        <v>372316245.14382505</v>
+      </c>
+      <c r="I8">
+        <v>205567448.85062256</v>
+      </c>
+      <c r="J8">
+        <v>298724285.85194606</v>
+      </c>
+      <c r="K8">
+        <v>383933273.50239819</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9">
+        <v>335380421.76351452</v>
+      </c>
+      <c r="C9">
+        <v>362352073.69339001</v>
+      </c>
+      <c r="D9">
+        <v>383520489.45837486</v>
+      </c>
+      <c r="E9">
+        <v>355784505.79011428</v>
+      </c>
+      <c r="F9">
+        <v>336875789.90134251</v>
+      </c>
+      <c r="G9">
+        <v>375014097.12652254</v>
+      </c>
+      <c r="H9">
+        <v>311718159.64401805</v>
+      </c>
+      <c r="I9">
+        <v>342118009.78200078</v>
+      </c>
+      <c r="J9">
+        <v>414126758.56879514</v>
+      </c>
+      <c r="K9">
+        <v>435582352.01399809</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10">
+        <v>549827474.98132467</v>
+      </c>
+      <c r="C10">
+        <v>665784401.94318473</v>
+      </c>
+      <c r="D10">
+        <v>727810488.02375126</v>
+      </c>
+      <c r="E10">
+        <v>817569325.23359919</v>
+      </c>
+      <c r="F10">
+        <v>591920647.62442482</v>
+      </c>
+      <c r="G10">
+        <v>644646003.95080864</v>
+      </c>
+      <c r="H10">
+        <v>735658958.48703182</v>
+      </c>
+      <c r="I10">
+        <v>1027608542.4071009</v>
+      </c>
+      <c r="J10">
+        <v>892550133.40725327</v>
+      </c>
+      <c r="K10">
+        <v>1074759377.9489493</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11">
+        <v>31963266.345840931</v>
+      </c>
+      <c r="C11">
+        <v>35039977.098894805</v>
+      </c>
+      <c r="D11">
+        <v>35258738.193920977</v>
+      </c>
+      <c r="E11">
+        <v>44894013.807144977</v>
+      </c>
+      <c r="F11">
+        <v>59200200.658337355</v>
+      </c>
+      <c r="G11">
+        <v>58897630.377025262</v>
+      </c>
+      <c r="H11">
+        <v>77401304.102025077</v>
+      </c>
+      <c r="I11">
+        <v>64631485.711945586</v>
+      </c>
+      <c r="J11">
+        <v>69982446.745643422</v>
+      </c>
+      <c r="K11">
+        <v>96407775.415615529</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>1</v>
+      </c>
+      <c r="B12">
+        <v>228897439.3742969</v>
+      </c>
+      <c r="C12">
+        <v>253779998.53891668</v>
+      </c>
+      <c r="D12">
+        <v>347563875.44835955</v>
+      </c>
+      <c r="E12">
+        <v>126077990.6876972</v>
+      </c>
+      <c r="F12">
+        <v>339611072.42515182</v>
+      </c>
+      <c r="G12">
+        <v>402374577.12272424</v>
+      </c>
+      <c r="H12">
+        <v>772673227.14698744</v>
+      </c>
+      <c r="I12">
+        <v>425391343.45268345</v>
+      </c>
+      <c r="J12">
+        <v>926810929.56272483</v>
+      </c>
+      <c r="K12">
+        <v>962534156.48327637</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B13">
+        <v>243363092.82996181</v>
+      </c>
+      <c r="C13">
+        <v>303936532.15251517</v>
+      </c>
+      <c r="D13">
+        <v>200898755.51546949</v>
+      </c>
+      <c r="E13">
+        <v>361957778.15674275</v>
+      </c>
+      <c r="F13">
+        <v>377486948.16756058</v>
+      </c>
+      <c r="G13">
+        <v>447683674.68108773</v>
+      </c>
+      <c r="H13">
+        <v>436557674.24829775</v>
+      </c>
+      <c r="I13">
+        <v>382900408.95075959</v>
+      </c>
+      <c r="J13">
+        <v>532200383.29412472</v>
+      </c>
+      <c r="K13">
+        <v>307477317.55869132</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0146DC9-AFE6-4966-A495-AA3F6F45C708}">
   <dimension ref="A1:K13"/>
@@ -2753,4 +3220,1852 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3A94711-7697-4899-A811-9A9EF746E2F9}">
+  <dimension ref="A1:K13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B1">
+        <v>1</v>
+      </c>
+      <c r="C1">
+        <v>2</v>
+      </c>
+      <c r="D1">
+        <v>3</v>
+      </c>
+      <c r="E1">
+        <v>4</v>
+      </c>
+      <c r="F1">
+        <v>5</v>
+      </c>
+      <c r="G1">
+        <v>6</v>
+      </c>
+      <c r="H1">
+        <v>7</v>
+      </c>
+      <c r="I1">
+        <v>8</v>
+      </c>
+      <c r="J1">
+        <v>9</v>
+      </c>
+      <c r="K1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2">
+        <v>247261081.24249551</v>
+      </c>
+      <c r="C2">
+        <v>759607940.76471853</v>
+      </c>
+      <c r="D2">
+        <v>332113816.48865902</v>
+      </c>
+      <c r="E2">
+        <v>518138302.12047517</v>
+      </c>
+      <c r="F2">
+        <v>554437574.5724448</v>
+      </c>
+      <c r="G2">
+        <v>1150395608.1171062</v>
+      </c>
+      <c r="H2">
+        <v>1252131858.0690684</v>
+      </c>
+      <c r="I2">
+        <v>624697356.39189005</v>
+      </c>
+      <c r="J2">
+        <v>1094661749.2913013</v>
+      </c>
+      <c r="K2">
+        <v>855920734.28939009</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>15606210.17351607</v>
+      </c>
+      <c r="C3">
+        <v>47723828.221244819</v>
+      </c>
+      <c r="D3">
+        <v>35682725.373119175</v>
+      </c>
+      <c r="E3">
+        <v>24215942.965926338</v>
+      </c>
+      <c r="F3">
+        <v>27124666.537699401</v>
+      </c>
+      <c r="G3">
+        <v>55229004.583887704</v>
+      </c>
+      <c r="H3">
+        <v>76110231.565105379</v>
+      </c>
+      <c r="I3">
+        <v>70366496.870226696</v>
+      </c>
+      <c r="J3">
+        <v>75970636.371245027</v>
+      </c>
+      <c r="K3">
+        <v>68581672.373427823</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
+        <v>190948844.07116279</v>
+      </c>
+      <c r="C4">
+        <v>480218476.69495869</v>
+      </c>
+      <c r="D4">
+        <v>151311679.9446007</v>
+      </c>
+      <c r="E4">
+        <v>718888423.53006554</v>
+      </c>
+      <c r="F4">
+        <v>560601786.49651611</v>
+      </c>
+      <c r="G4">
+        <v>579803075.07805192</v>
+      </c>
+      <c r="H4">
+        <v>282882381.32612872</v>
+      </c>
+      <c r="I4">
+        <v>876939583.63994825</v>
+      </c>
+      <c r="J4">
+        <v>981721441.50337565</v>
+      </c>
+      <c r="K4">
+        <v>883337836.43675768</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5">
+        <v>545886518.23867655</v>
+      </c>
+      <c r="C5">
+        <v>902179583.3433063</v>
+      </c>
+      <c r="D5">
+        <v>999330445.97705555</v>
+      </c>
+      <c r="E5">
+        <v>757282085.98983467</v>
+      </c>
+      <c r="F5">
+        <v>506359586.79327196</v>
+      </c>
+      <c r="G5">
+        <v>1070957210.5827363</v>
+      </c>
+      <c r="H5">
+        <v>1320737437.4398692</v>
+      </c>
+      <c r="I5">
+        <v>1061491908.2184124</v>
+      </c>
+      <c r="J5">
+        <v>1765243172.2341905</v>
+      </c>
+      <c r="K5">
+        <v>1528314439.8217499</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6">
+        <v>625144487.81632018</v>
+      </c>
+      <c r="C6">
+        <v>599688733.60756576</v>
+      </c>
+      <c r="D6">
+        <v>700173776.81375015</v>
+      </c>
+      <c r="E6">
+        <v>698617201.06906307</v>
+      </c>
+      <c r="F6">
+        <v>852703034.15588212</v>
+      </c>
+      <c r="G6">
+        <v>677166605.81659639</v>
+      </c>
+      <c r="H6">
+        <v>694384671.86013925</v>
+      </c>
+      <c r="I6">
+        <v>682155742.12745571</v>
+      </c>
+      <c r="J6">
+        <v>746439858.05037344</v>
+      </c>
+      <c r="K6">
+        <v>637038012.07378983</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>388529421.86720604</v>
+      </c>
+      <c r="C7">
+        <v>297220409.07591468</v>
+      </c>
+      <c r="D7">
+        <v>352699883.36336654</v>
+      </c>
+      <c r="E7">
+        <v>368334295.42635912</v>
+      </c>
+      <c r="F7">
+        <v>374772798.61739916</v>
+      </c>
+      <c r="G7">
+        <v>381311717.42835397</v>
+      </c>
+      <c r="H7">
+        <v>326518967.16641867</v>
+      </c>
+      <c r="I7">
+        <v>400697649.30417931</v>
+      </c>
+      <c r="J7">
+        <v>461291239.52330929</v>
+      </c>
+      <c r="K7">
+        <v>442600788.28196692</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8">
+        <v>449867903.82097661</v>
+      </c>
+      <c r="C8">
+        <v>284172162.19225121</v>
+      </c>
+      <c r="D8">
+        <v>419715536.61845392</v>
+      </c>
+      <c r="E8">
+        <v>394409077.00138319</v>
+      </c>
+      <c r="F8">
+        <v>304551679.59428209</v>
+      </c>
+      <c r="G8">
+        <v>442069065.93475425</v>
+      </c>
+      <c r="H8">
+        <v>533082193.12995094</v>
+      </c>
+      <c r="I8">
+        <v>503458397.19650191</v>
+      </c>
+      <c r="J8">
+        <v>110062834.5576396</v>
+      </c>
+      <c r="K8">
+        <v>485385348.01318401</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9">
+        <v>317444591.46364534</v>
+      </c>
+      <c r="C9">
+        <v>330104270.74600965</v>
+      </c>
+      <c r="D9">
+        <v>278319090.76157832</v>
+      </c>
+      <c r="E9">
+        <v>309337323.47656822</v>
+      </c>
+      <c r="F9">
+        <v>333919044.5213623</v>
+      </c>
+      <c r="G9">
+        <v>405223999.12006789</v>
+      </c>
+      <c r="H9">
+        <v>384109310.00471282</v>
+      </c>
+      <c r="I9">
+        <v>413772316.68779159</v>
+      </c>
+      <c r="J9">
+        <v>399412018.89954674</v>
+      </c>
+      <c r="K9">
+        <v>445230150.92320961</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10">
+        <v>549827474.98132467</v>
+      </c>
+      <c r="C10">
+        <v>649335475.72061336</v>
+      </c>
+      <c r="D10">
+        <v>665345140.96517253</v>
+      </c>
+      <c r="E10">
+        <v>626073557.34464645</v>
+      </c>
+      <c r="F10">
+        <v>785723057.96659529</v>
+      </c>
+      <c r="G10">
+        <v>821768160.56431961</v>
+      </c>
+      <c r="H10">
+        <v>1063990468.3855669</v>
+      </c>
+      <c r="I10">
+        <v>865082172.11767256</v>
+      </c>
+      <c r="J10">
+        <v>830759601.32490122</v>
+      </c>
+      <c r="K10">
+        <v>1150976471.7755027</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11">
+        <v>31963266.345840931</v>
+      </c>
+      <c r="C11">
+        <v>33375292.227423828</v>
+      </c>
+      <c r="D11">
+        <v>39201568.523249254</v>
+      </c>
+      <c r="E11">
+        <v>42542337.141828336</v>
+      </c>
+      <c r="F11">
+        <v>46477805.033111945</v>
+      </c>
+      <c r="G11">
+        <v>53015293.319497779</v>
+      </c>
+      <c r="H11">
+        <v>67233139.407706693</v>
+      </c>
+      <c r="I11">
+        <v>81140345.884170264</v>
+      </c>
+      <c r="J11">
+        <v>78095127.904564857</v>
+      </c>
+      <c r="K11">
+        <v>87600084.422066689</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>1</v>
+      </c>
+      <c r="B12">
+        <v>208241169.07629019</v>
+      </c>
+      <c r="C12">
+        <v>288904036.91733217</v>
+      </c>
+      <c r="D12">
+        <v>344797452.17013919</v>
+      </c>
+      <c r="E12">
+        <v>432242643.81074345</v>
+      </c>
+      <c r="F12">
+        <v>399356804.62830859</v>
+      </c>
+      <c r="G12">
+        <v>373798073.11991167</v>
+      </c>
+      <c r="H12">
+        <v>484149045.40093631</v>
+      </c>
+      <c r="I12">
+        <v>558128063.34938288</v>
+      </c>
+      <c r="J12">
+        <v>704125074.68157959</v>
+      </c>
+      <c r="K12">
+        <v>873263171.80820048</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B13">
+        <v>211403260.01881739</v>
+      </c>
+      <c r="C13">
+        <v>228329818.85721302</v>
+      </c>
+      <c r="D13">
+        <v>235475582.84448794</v>
+      </c>
+      <c r="E13">
+        <v>260513581.63570553</v>
+      </c>
+      <c r="F13">
+        <v>435269936.97858447</v>
+      </c>
+      <c r="G13">
+        <v>300403696.99465197</v>
+      </c>
+      <c r="H13">
+        <v>392943930.8031829</v>
+      </c>
+      <c r="I13">
+        <v>314206243.35590744</v>
+      </c>
+      <c r="J13">
+        <v>381872485.6863296</v>
+      </c>
+      <c r="K13">
+        <v>522515223.11309469</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EFAD5CC-841F-420F-81CE-DF72BE77F0F0}">
+  <dimension ref="A1:K13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B1">
+        <v>1</v>
+      </c>
+      <c r="C1">
+        <v>2</v>
+      </c>
+      <c r="D1">
+        <v>3</v>
+      </c>
+      <c r="E1">
+        <v>4</v>
+      </c>
+      <c r="F1">
+        <v>5</v>
+      </c>
+      <c r="G1">
+        <v>6</v>
+      </c>
+      <c r="H1">
+        <v>7</v>
+      </c>
+      <c r="I1">
+        <v>8</v>
+      </c>
+      <c r="J1">
+        <v>9</v>
+      </c>
+      <c r="K1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2">
+        <v>668711630.97059476</v>
+      </c>
+      <c r="C2">
+        <v>343669936.59644687</v>
+      </c>
+      <c r="D2">
+        <v>174825189.23867741</v>
+      </c>
+      <c r="E2">
+        <v>539989639.53772116</v>
+      </c>
+      <c r="F2">
+        <v>1091759871.9047999</v>
+      </c>
+      <c r="G2">
+        <v>427571662.35059226</v>
+      </c>
+      <c r="H2">
+        <v>639432535.25970995</v>
+      </c>
+      <c r="I2">
+        <v>757357256.86270702</v>
+      </c>
+      <c r="J2">
+        <v>654910312.09929729</v>
+      </c>
+      <c r="K2">
+        <v>1280587543.8287516</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>37312113.854833707</v>
+      </c>
+      <c r="C3">
+        <v>34883890.082127385</v>
+      </c>
+      <c r="D3">
+        <v>35093612.029788196</v>
+      </c>
+      <c r="E3">
+        <v>44035962.055731349</v>
+      </c>
+      <c r="F3">
+        <v>5745642.3871950284</v>
+      </c>
+      <c r="G3">
+        <v>50091480.098307639</v>
+      </c>
+      <c r="H3">
+        <v>46881165.302780442</v>
+      </c>
+      <c r="I3">
+        <v>59133925.922221959</v>
+      </c>
+      <c r="J3">
+        <v>95831762.700491905</v>
+      </c>
+      <c r="K3">
+        <v>68629482.563776448</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
+        <v>239727364.35040218</v>
+      </c>
+      <c r="C4">
+        <v>330454848.71202046</v>
+      </c>
+      <c r="D4">
+        <v>444419619.44191033</v>
+      </c>
+      <c r="E4">
+        <v>144568843.93537959</v>
+      </c>
+      <c r="F4">
+        <v>510923291.91265082</v>
+      </c>
+      <c r="G4">
+        <v>481059337.83157074</v>
+      </c>
+      <c r="H4">
+        <v>786804205.54634356</v>
+      </c>
+      <c r="I4">
+        <v>1210843616.6671238</v>
+      </c>
+      <c r="J4">
+        <v>857237473.68598306</v>
+      </c>
+      <c r="K4">
+        <v>770378114.77987039</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5">
+        <v>545886518.23867655</v>
+      </c>
+      <c r="C5">
+        <v>732646291.66530013</v>
+      </c>
+      <c r="D5">
+        <v>923664204.47821128</v>
+      </c>
+      <c r="E5">
+        <v>1138101496.7281032</v>
+      </c>
+      <c r="F5">
+        <v>968071214.79522061</v>
+      </c>
+      <c r="G5">
+        <v>951414125.03952909</v>
+      </c>
+      <c r="H5">
+        <v>1319236575.0681725</v>
+      </c>
+      <c r="I5">
+        <v>2314298424.9203072</v>
+      </c>
+      <c r="J5">
+        <v>1099965808.5331051</v>
+      </c>
+      <c r="K5">
+        <v>1918543604.4199703</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6">
+        <v>570605073.91759527</v>
+      </c>
+      <c r="C6">
+        <v>752572987.22965991</v>
+      </c>
+      <c r="D6">
+        <v>609617462.40558064</v>
+      </c>
+      <c r="E6">
+        <v>800127009.68302965</v>
+      </c>
+      <c r="F6">
+        <v>498585680.4414829</v>
+      </c>
+      <c r="G6">
+        <v>598448270.89847481</v>
+      </c>
+      <c r="H6">
+        <v>557022992.22647822</v>
+      </c>
+      <c r="I6">
+        <v>728471691.43471515</v>
+      </c>
+      <c r="J6">
+        <v>603852699.80979085</v>
+      </c>
+      <c r="K6">
+        <v>641866107.35222507</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>329713634.04730356</v>
+      </c>
+      <c r="C7">
+        <v>297220409.07591468</v>
+      </c>
+      <c r="D7">
+        <v>406546045.32465708</v>
+      </c>
+      <c r="E7">
+        <v>372175457.82157648</v>
+      </c>
+      <c r="F7">
+        <v>408476004.36618936</v>
+      </c>
+      <c r="G7">
+        <v>311485773.28444356</v>
+      </c>
+      <c r="H7">
+        <v>331193439.03552932</v>
+      </c>
+      <c r="I7">
+        <v>398978528.72012931</v>
+      </c>
+      <c r="J7">
+        <v>404309514.7301743</v>
+      </c>
+      <c r="K7">
+        <v>378526812.06620282</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8">
+        <v>449867903.82097661</v>
+      </c>
+      <c r="C8">
+        <v>494109545.4175849</v>
+      </c>
+      <c r="D8">
+        <v>510206267.37118363</v>
+      </c>
+      <c r="E8">
+        <v>482769765.63309532</v>
+      </c>
+      <c r="F8">
+        <v>270889017.149517</v>
+      </c>
+      <c r="G8">
+        <v>382837060.66452962</v>
+      </c>
+      <c r="H8">
+        <v>360130151.846771</v>
+      </c>
+      <c r="I8">
+        <v>503118825.15352166</v>
+      </c>
+      <c r="J8">
+        <v>110062834.5576396</v>
+      </c>
+      <c r="K8">
+        <v>172974649.74818462</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9">
+        <v>335380421.76351452</v>
+      </c>
+      <c r="C9">
+        <v>350379877.2416085</v>
+      </c>
+      <c r="D9">
+        <v>373511233.6512301</v>
+      </c>
+      <c r="E9">
+        <v>367356224.8504656</v>
+      </c>
+      <c r="F9">
+        <v>351988642.34770811</v>
+      </c>
+      <c r="G9">
+        <v>314864778.13330781</v>
+      </c>
+      <c r="H9">
+        <v>373052819.82748193</v>
+      </c>
+      <c r="I9">
+        <v>385117009.53653872</v>
+      </c>
+      <c r="J9">
+        <v>424590012.74649632</v>
+      </c>
+      <c r="K9">
+        <v>511091696.20727473</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10">
+        <v>716469135.2208643</v>
+      </c>
+      <c r="C10">
+        <v>641690383.25495183</v>
+      </c>
+      <c r="D10">
+        <v>831324530.47489452</v>
+      </c>
+      <c r="E10">
+        <v>746199758.562837</v>
+      </c>
+      <c r="F10">
+        <v>978767909.04237306</v>
+      </c>
+      <c r="G10">
+        <v>784965883.20988262</v>
+      </c>
+      <c r="H10">
+        <v>872327444.27031887</v>
+      </c>
+      <c r="I10">
+        <v>942731154.56997395</v>
+      </c>
+      <c r="J10">
+        <v>933702627.21211207</v>
+      </c>
+      <c r="K10">
+        <v>1053409922.0494395</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11">
+        <v>25915770.51731832</v>
+      </c>
+      <c r="C11">
+        <v>35304408.818233117</v>
+      </c>
+      <c r="D11">
+        <v>37580051.914142713</v>
+      </c>
+      <c r="E11">
+        <v>43887672.600120068</v>
+      </c>
+      <c r="F11">
+        <v>55331655.701926373</v>
+      </c>
+      <c r="G11">
+        <v>63387767.790828109</v>
+      </c>
+      <c r="H11">
+        <v>75044622.674456492</v>
+      </c>
+      <c r="I11">
+        <v>79466980.161214933</v>
+      </c>
+      <c r="J11">
+        <v>78333669.233772039</v>
+      </c>
+      <c r="K11">
+        <v>103018506.59042895</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>1</v>
+      </c>
+      <c r="B12">
+        <v>239577204.00124341</v>
+      </c>
+      <c r="C12">
+        <v>136461943.51271439</v>
+      </c>
+      <c r="D12">
+        <v>298057034.35959572</v>
+      </c>
+      <c r="E12">
+        <v>458930348.94241369</v>
+      </c>
+      <c r="F12">
+        <v>416977937.66603076</v>
+      </c>
+      <c r="G12">
+        <v>282010394.88296014</v>
+      </c>
+      <c r="H12">
+        <v>634155260.80450094</v>
+      </c>
+      <c r="I12">
+        <v>745107668.75338006</v>
+      </c>
+      <c r="J12">
+        <v>672046970.92515421</v>
+      </c>
+      <c r="K12">
+        <v>568740774.64179826</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B13">
+        <v>252940083.3603006</v>
+      </c>
+      <c r="C13">
+        <v>303936532.15251517</v>
+      </c>
+      <c r="D13">
+        <v>200898755.51546949</v>
+      </c>
+      <c r="E13">
+        <v>235491346.20729747</v>
+      </c>
+      <c r="F13">
+        <v>354997830.73208255</v>
+      </c>
+      <c r="G13">
+        <v>306546004.95659447</v>
+      </c>
+      <c r="H13">
+        <v>368763357.99411893</v>
+      </c>
+      <c r="I13">
+        <v>551890904.61242998</v>
+      </c>
+      <c r="J13">
+        <v>570312461.74151504</v>
+      </c>
+      <c r="K13">
+        <v>462516930.16248465</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E53E8DB-A824-4746-8747-6D57876EB982}">
+  <dimension ref="A1:K13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B1">
+        <v>1</v>
+      </c>
+      <c r="C1">
+        <v>2</v>
+      </c>
+      <c r="D1">
+        <v>3</v>
+      </c>
+      <c r="E1">
+        <v>4</v>
+      </c>
+      <c r="F1">
+        <v>5</v>
+      </c>
+      <c r="G1">
+        <v>6</v>
+      </c>
+      <c r="H1">
+        <v>7</v>
+      </c>
+      <c r="I1">
+        <v>8</v>
+      </c>
+      <c r="J1">
+        <v>9</v>
+      </c>
+      <c r="K1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2">
+        <v>518256994.77674192</v>
+      </c>
+      <c r="C2">
+        <v>602000961.33807218</v>
+      </c>
+      <c r="D2">
+        <v>174825189.23867741</v>
+      </c>
+      <c r="E2">
+        <v>868019126.67763531</v>
+      </c>
+      <c r="F2">
+        <v>1163611429.679358</v>
+      </c>
+      <c r="G2">
+        <v>418777197.47336662</v>
+      </c>
+      <c r="H2">
+        <v>380299767.14367753</v>
+      </c>
+      <c r="I2">
+        <v>503855545.62899768</v>
+      </c>
+      <c r="J2">
+        <v>691028200.5669378</v>
+      </c>
+      <c r="K2">
+        <v>828606213.02712369</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>32754558.748005256</v>
+      </c>
+      <c r="C3">
+        <v>20506877.034425657</v>
+      </c>
+      <c r="D3">
+        <v>23918106.814861406</v>
+      </c>
+      <c r="E3">
+        <v>40835291.222810224</v>
+      </c>
+      <c r="F3">
+        <v>27427938.970678993</v>
+      </c>
+      <c r="G3">
+        <v>26761914.765856057</v>
+      </c>
+      <c r="H3">
+        <v>45101628.894908458</v>
+      </c>
+      <c r="I3">
+        <v>70128209.067125633</v>
+      </c>
+      <c r="J3">
+        <v>85531913.65493153</v>
+      </c>
+      <c r="K3">
+        <v>66213714.655984484</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
+        <v>351512825.04188097</v>
+      </c>
+      <c r="C4">
+        <v>581735022.12455821</v>
+      </c>
+      <c r="D4">
+        <v>609953511.51645839</v>
+      </c>
+      <c r="E4">
+        <v>833845846.65265334</v>
+      </c>
+      <c r="F4">
+        <v>935183993.09773898</v>
+      </c>
+      <c r="G4">
+        <v>528973789.1498552</v>
+      </c>
+      <c r="H4">
+        <v>522628676.88023853</v>
+      </c>
+      <c r="I4">
+        <v>596914038.62396407</v>
+      </c>
+      <c r="J4">
+        <v>235150244.26045865</v>
+      </c>
+      <c r="K4">
+        <v>912030875.05791473</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5">
+        <v>777076702.64843607</v>
+      </c>
+      <c r="C5">
+        <v>902179583.3433063</v>
+      </c>
+      <c r="D5">
+        <v>799645417.55604863</v>
+      </c>
+      <c r="E5">
+        <v>557160172.62881207</v>
+      </c>
+      <c r="F5">
+        <v>693021882.52332282</v>
+      </c>
+      <c r="G5">
+        <v>1217934971.0723619</v>
+      </c>
+      <c r="H5">
+        <v>1496484767.7350633</v>
+      </c>
+      <c r="I5">
+        <v>1247075707.8154938</v>
+      </c>
+      <c r="J5">
+        <v>895035270.24537349</v>
+      </c>
+      <c r="K5">
+        <v>2480490989.6650343</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6">
+        <v>712021988.8411392</v>
+      </c>
+      <c r="C6">
+        <v>752572987.22965991</v>
+      </c>
+      <c r="D6">
+        <v>602278887.59809768</v>
+      </c>
+      <c r="E6">
+        <v>577384620.42296469</v>
+      </c>
+      <c r="F6">
+        <v>753654076.18370879</v>
+      </c>
+      <c r="G6">
+        <v>689461464.9778862</v>
+      </c>
+      <c r="H6">
+        <v>562750881.6833595</v>
+      </c>
+      <c r="I6">
+        <v>754819814.46898127</v>
+      </c>
+      <c r="J6">
+        <v>809862206.63056946</v>
+      </c>
+      <c r="K6">
+        <v>833516667.99908423</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>313184875.6168254</v>
+      </c>
+      <c r="C7">
+        <v>359930250.1071701</v>
+      </c>
+      <c r="D7">
+        <v>314439966.41080499</v>
+      </c>
+      <c r="E7">
+        <v>274333558.66616201</v>
+      </c>
+      <c r="F7">
+        <v>471001453.41055518</v>
+      </c>
+      <c r="G7">
+        <v>325442212.39754474</v>
+      </c>
+      <c r="H7">
+        <v>399623736.0700509</v>
+      </c>
+      <c r="I7">
+        <v>485205389.93615353</v>
+      </c>
+      <c r="J7">
+        <v>369637826.72381473</v>
+      </c>
+      <c r="K7">
+        <v>398893844.48378503</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8">
+        <v>355535773.25645244</v>
+      </c>
+      <c r="C8">
+        <v>494109545.4175849</v>
+      </c>
+      <c r="D8">
+        <v>411083621.8428793</v>
+      </c>
+      <c r="E8">
+        <v>480114577.87666106</v>
+      </c>
+      <c r="F8">
+        <v>269631817.47397655</v>
+      </c>
+      <c r="G8">
+        <v>417025639.09656298</v>
+      </c>
+      <c r="H8">
+        <v>516322367.41152835</v>
+      </c>
+      <c r="I8">
+        <v>370147630.7617594</v>
+      </c>
+      <c r="J8">
+        <v>624924180.90357208</v>
+      </c>
+      <c r="K8">
+        <v>382070699.48055875</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9">
+        <v>269139832.50298101</v>
+      </c>
+      <c r="C9">
+        <v>281693484.01241022</v>
+      </c>
+      <c r="D9">
+        <v>355574244.31334835</v>
+      </c>
+      <c r="E9">
+        <v>335673557.64857292</v>
+      </c>
+      <c r="F9">
+        <v>384146890.0618428</v>
+      </c>
+      <c r="G9">
+        <v>372895439.9614833</v>
+      </c>
+      <c r="H9">
+        <v>405777479.6031093</v>
+      </c>
+      <c r="I9">
+        <v>458282668.86248535</v>
+      </c>
+      <c r="J9">
+        <v>400777950.64928144</v>
+      </c>
+      <c r="K9">
+        <v>464227135.32589775</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10">
+        <v>611416953.3747375</v>
+      </c>
+      <c r="C10">
+        <v>783694552.35479057</v>
+      </c>
+      <c r="D10">
+        <v>667812724.05628729</v>
+      </c>
+      <c r="E10">
+        <v>519253104.41226047</v>
+      </c>
+      <c r="F10">
+        <v>590364564.66679251</v>
+      </c>
+      <c r="G10">
+        <v>709257313.73606312</v>
+      </c>
+      <c r="H10">
+        <v>694714246.66252828</v>
+      </c>
+      <c r="I10">
+        <v>786910089.96954679</v>
+      </c>
+      <c r="J10">
+        <v>951532991.62052488</v>
+      </c>
+      <c r="K10">
+        <v>765512797.18777096</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11">
+        <v>25915770.51731832</v>
+      </c>
+      <c r="C11">
+        <v>33357791.382223364</v>
+      </c>
+      <c r="D11">
+        <v>43657788.688030601</v>
+      </c>
+      <c r="E11">
+        <v>50490572.91107028</v>
+      </c>
+      <c r="F11">
+        <v>57034492.867158569</v>
+      </c>
+      <c r="G11">
+        <v>50636624.036284722</v>
+      </c>
+      <c r="H11">
+        <v>66658868.24270916</v>
+      </c>
+      <c r="I11">
+        <v>70543470.4331384</v>
+      </c>
+      <c r="J11">
+        <v>77520547.353202909</v>
+      </c>
+      <c r="K11">
+        <v>85177288.541013971</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>1</v>
+      </c>
+      <c r="B12">
+        <v>219350873.51259035</v>
+      </c>
+      <c r="C12">
+        <v>288904036.91733217</v>
+      </c>
+      <c r="D12">
+        <v>176538090.23275802</v>
+      </c>
+      <c r="E12">
+        <v>253103362.40070152</v>
+      </c>
+      <c r="F12">
+        <v>287956465.49230486</v>
+      </c>
+      <c r="G12">
+        <v>566243423.6995163</v>
+      </c>
+      <c r="H12">
+        <v>484780965.24311888</v>
+      </c>
+      <c r="I12">
+        <v>543754907.43233669</v>
+      </c>
+      <c r="J12">
+        <v>632271952.77963912</v>
+      </c>
+      <c r="K12">
+        <v>608229485.4154191</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B13">
+        <v>211403260.01881739</v>
+      </c>
+      <c r="C13">
+        <v>290007823.87345493</v>
+      </c>
+      <c r="D13">
+        <v>342684570.96505648</v>
+      </c>
+      <c r="E13">
+        <v>188469763.52293101</v>
+      </c>
+      <c r="F13">
+        <v>174864390.95097542</v>
+      </c>
+      <c r="G13">
+        <v>153059748.41270599</v>
+      </c>
+      <c r="H13">
+        <v>427262025.38911951</v>
+      </c>
+      <c r="I13">
+        <v>212857467.72997287</v>
+      </c>
+      <c r="J13">
+        <v>536335443.54594374</v>
+      </c>
+      <c r="K13">
+        <v>567947903.91551626</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D7B5E39-262B-427E-BF30-8FCF23F0B28A}">
+  <dimension ref="A1:K13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B1">
+        <v>1</v>
+      </c>
+      <c r="C1">
+        <v>2</v>
+      </c>
+      <c r="D1">
+        <v>3</v>
+      </c>
+      <c r="E1">
+        <v>4</v>
+      </c>
+      <c r="F1">
+        <v>5</v>
+      </c>
+      <c r="G1">
+        <v>6</v>
+      </c>
+      <c r="H1">
+        <v>7</v>
+      </c>
+      <c r="I1">
+        <v>8</v>
+      </c>
+      <c r="J1">
+        <v>9</v>
+      </c>
+      <c r="K1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2">
+        <v>526291191.84850961</v>
+      </c>
+      <c r="C2">
+        <v>477137571.52775073</v>
+      </c>
+      <c r="D2">
+        <v>174825189.23867741</v>
+      </c>
+      <c r="E2">
+        <v>491237729.7406168</v>
+      </c>
+      <c r="F2">
+        <v>928458518.48427606</v>
+      </c>
+      <c r="G2">
+        <v>692050910.39959645</v>
+      </c>
+      <c r="H2">
+        <v>497569901.36802095</v>
+      </c>
+      <c r="I2">
+        <v>458436025.33761138</v>
+      </c>
+      <c r="J2">
+        <v>415797066.36775917</v>
+      </c>
+      <c r="K2">
+        <v>1197950900.9301076</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>15606210.17351607</v>
+      </c>
+      <c r="C3">
+        <v>11550680.10724384</v>
+      </c>
+      <c r="D3">
+        <v>8463058.944489466</v>
+      </c>
+      <c r="E3">
+        <v>64308511.223516516</v>
+      </c>
+      <c r="F3">
+        <v>58293451.609304652</v>
+      </c>
+      <c r="G3">
+        <v>82882131.858521789</v>
+      </c>
+      <c r="H3">
+        <v>47948179.287704095</v>
+      </c>
+      <c r="I3">
+        <v>22972717.255909901</v>
+      </c>
+      <c r="J3">
+        <v>29283769.417316139</v>
+      </c>
+      <c r="K3">
+        <v>90854356.617164999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
+        <v>305460979.94083011</v>
+      </c>
+      <c r="C4">
+        <v>158982392.35144421</v>
+      </c>
+      <c r="D4">
+        <v>288426287.36909765</v>
+      </c>
+      <c r="E4">
+        <v>337624288.72328377</v>
+      </c>
+      <c r="F4">
+        <v>456533465.89998585</v>
+      </c>
+      <c r="G4">
+        <v>542357008.81245375</v>
+      </c>
+      <c r="H4">
+        <v>633789616.46441245</v>
+      </c>
+      <c r="I4">
+        <v>701363534.65947628</v>
+      </c>
+      <c r="J4">
+        <v>900329933.62878966</v>
+      </c>
+      <c r="K4">
+        <v>971580356.29452384</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5">
+        <v>545886518.23867655</v>
+      </c>
+      <c r="C5">
+        <v>902179583.3433063</v>
+      </c>
+      <c r="D5">
+        <v>1048139752.510308</v>
+      </c>
+      <c r="E5">
+        <v>484972305.39345986</v>
+      </c>
+      <c r="F5">
+        <v>869013118.30558991</v>
+      </c>
+      <c r="G5">
+        <v>1160393982.3016529</v>
+      </c>
+      <c r="H5">
+        <v>1245330136.8621011</v>
+      </c>
+      <c r="I5">
+        <v>906468544.05628872</v>
+      </c>
+      <c r="J5">
+        <v>2176556596.7335682</v>
+      </c>
+      <c r="K5">
+        <v>1818279716.8689728</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6">
+        <v>578754437.13347745</v>
+      </c>
+      <c r="C6">
+        <v>590235012.8700428</v>
+      </c>
+      <c r="D6">
+        <v>686338366.68517065</v>
+      </c>
+      <c r="E6">
+        <v>692181756.9853251</v>
+      </c>
+      <c r="F6">
+        <v>739789250.55462217</v>
+      </c>
+      <c r="G6">
+        <v>624132946.7349683</v>
+      </c>
+      <c r="H6">
+        <v>774434529.95757699</v>
+      </c>
+      <c r="I6">
+        <v>689573010.71967793</v>
+      </c>
+      <c r="J6">
+        <v>645159204.98187327</v>
+      </c>
+      <c r="K6">
+        <v>908285010.93987703</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>361274010.58396024</v>
+      </c>
+      <c r="C7">
+        <v>357071201.70787102</v>
+      </c>
+      <c r="D7">
+        <v>284867436.90863109</v>
+      </c>
+      <c r="E7">
+        <v>352336010.48216367</v>
+      </c>
+      <c r="F7">
+        <v>382578904.06145048</v>
+      </c>
+      <c r="G7">
+        <v>457836961.82619268</v>
+      </c>
+      <c r="H7">
+        <v>394446564.37970591</v>
+      </c>
+      <c r="I7">
+        <v>397884596.3586188</v>
+      </c>
+      <c r="J7">
+        <v>490012636.25782585</v>
+      </c>
+      <c r="K7">
+        <v>339658108.68351215</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8">
+        <v>313064095.43054122</v>
+      </c>
+      <c r="C8">
+        <v>284172162.19225121</v>
+      </c>
+      <c r="D8">
+        <v>450859599.92730314</v>
+      </c>
+      <c r="E8">
+        <v>572403616.95103526</v>
+      </c>
+      <c r="F8">
+        <v>563914688.2460115</v>
+      </c>
+      <c r="G8">
+        <v>480651110.34809339</v>
+      </c>
+      <c r="H8">
+        <v>593380411.40304422</v>
+      </c>
+      <c r="I8">
+        <v>292406052.59223086</v>
+      </c>
+      <c r="J8">
+        <v>394559228.51278597</v>
+      </c>
+      <c r="K8">
+        <v>464119435.7112323</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9">
+        <v>305366404.75257719</v>
+      </c>
+      <c r="C9">
+        <v>316869347.75238496</v>
+      </c>
+      <c r="D9">
+        <v>264264474.10539895</v>
+      </c>
+      <c r="E9">
+        <v>343746594.08753127</v>
+      </c>
+      <c r="F9">
+        <v>325386900.72814471</v>
+      </c>
+      <c r="G9">
+        <v>358509604.90765285</v>
+      </c>
+      <c r="H9">
+        <v>358318010.06093246</v>
+      </c>
+      <c r="I9">
+        <v>351403913.04201114</v>
+      </c>
+      <c r="J9">
+        <v>404943942.49745566</v>
+      </c>
+      <c r="K9">
+        <v>419478510.16289997</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10">
+        <v>549827474.98132467</v>
+      </c>
+      <c r="C10">
+        <v>783032286.5220927</v>
+      </c>
+      <c r="D10">
+        <v>847853208.89578772</v>
+      </c>
+      <c r="E10">
+        <v>792128886.07483399</v>
+      </c>
+      <c r="F10">
+        <v>798888095.95721853</v>
+      </c>
+      <c r="G10">
+        <v>753979141.1861968</v>
+      </c>
+      <c r="H10">
+        <v>956844648.43030322</v>
+      </c>
+      <c r="I10">
+        <v>668010806.46001875</v>
+      </c>
+      <c r="J10">
+        <v>862121946.63611412</v>
+      </c>
+      <c r="K10">
+        <v>979626235.46349871</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11">
+        <v>27221843.135823727</v>
+      </c>
+      <c r="C11">
+        <v>37560596.829000391</v>
+      </c>
+      <c r="D11">
+        <v>38472210.079991974</v>
+      </c>
+      <c r="E11">
+        <v>48393703.268619008</v>
+      </c>
+      <c r="F11">
+        <v>58491597.171470471</v>
+      </c>
+      <c r="G11">
+        <v>67306672.186233982</v>
+      </c>
+      <c r="H11">
+        <v>66245822.319170363</v>
+      </c>
+      <c r="I11">
+        <v>80099093.641012266</v>
+      </c>
+      <c r="J11">
+        <v>80603310.368913084</v>
+      </c>
+      <c r="K11">
+        <v>87491929.594395205</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>1</v>
+      </c>
+      <c r="B12">
+        <v>191466627.26020518</v>
+      </c>
+      <c r="C12">
+        <v>269759327.45659679</v>
+      </c>
+      <c r="D12">
+        <v>370114448.41798627</v>
+      </c>
+      <c r="E12">
+        <v>222645068.45803604</v>
+      </c>
+      <c r="F12">
+        <v>399497383.25196576</v>
+      </c>
+      <c r="G12">
+        <v>363331552.33162981</v>
+      </c>
+      <c r="H12">
+        <v>604824479.94275045</v>
+      </c>
+      <c r="I12">
+        <v>456702953.37521821</v>
+      </c>
+      <c r="J12">
+        <v>690759677.01812208</v>
+      </c>
+      <c r="K12">
+        <v>627013464.95231831</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B13">
+        <v>252940083.3603006</v>
+      </c>
+      <c r="C13">
+        <v>208856647.25570789</v>
+      </c>
+      <c r="D13">
+        <v>270904887.16533935</v>
+      </c>
+      <c r="E13">
+        <v>392954090.38451391</v>
+      </c>
+      <c r="F13">
+        <v>268288986.45660722</v>
+      </c>
+      <c r="G13">
+        <v>301970786.90467227</v>
+      </c>
+      <c r="H13">
+        <v>437058511.69763005</v>
+      </c>
+      <c r="I13">
+        <v>451689738.09964168</v>
+      </c>
+      <c r="J13">
+        <v>359249462.48754233</v>
+      </c>
+      <c r="K13">
+        <v>271206507.68901116</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>